<commit_message>
Verifica la nota 554 (Ryle, p. 19); no quedan notas pendientes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JFqB7qFXyXBvPWdV8axcUP
</commit_message>
<xml_diff>
--- a/Verificacion_citas_Cap_III.xlsx
+++ b/Verificacion_citas_Cap_III.xlsx
@@ -571,7 +571,7 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>174</v>
+        <v>175</v>
       </c>
     </row>
     <row r="9">
@@ -601,7 +601,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -638,7 +638,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>(1) SUP-JIN-194/2025: el voto de Rodríguez Mondragón y su proyecto se cotejaron con el PDF en tramos (40-120, 121-200 y 200-300) que el usuario puso a disposición. En ese documento varias hojas tienen el número impreso fuera de orden (21 antes que 20, 91 antes que 90, 101 antes que 100, etc.); se siguió el número impreso de cada hoja, que es el que usa la tesis. (2) Ryle, The Concept of Mind: se recibieron las pp. 13-18; la nota 554 (p. 19) queda pendiente.</t>
+          <t>SUP-JIN-194/2025: el voto de Rodríguez Mondragón y su proyecto se cotejaron con el PDF en tramos (40-120, 121-200 y 200-300). En ese documento varias hojas tienen el número impreso fuera de orden (21 antes que 20, 91 antes que 90, 101 antes que 100, etc.); se siguió el número impreso de cada hoja, que es el que usa la tesis. Ryle se cotejó con las pp. 13-19 enviadas por el usuario.</t>
         </is>
       </c>
     </row>
@@ -9230,14 +9230,14 @@
           <t>The Concept of Mind (pp. 13-18 subidas por el usuario)</t>
         </is>
       </c>
-      <c r="H185" s="6" t="inlineStr">
-        <is>
-          <t>Pendiente (fuente no disponible)</t>
+      <c r="H185" s="3" t="inlineStr">
+        <is>
+          <t>Conforme</t>
         </is>
       </c>
       <c r="I185" s="2" t="inlineStr">
         <is>
-          <t>Ryle, p. 19: el archivo subido abarca las pp. 13-18; la p. 18 termina con el ejemplo del críquet y el pasaje citado debe seguir en la p. 19, que no se recibió.</t>
+          <t>Ryle, The Concept of Mind, p. 19 (imagen enviada por el usuario): «The theoretically interesting category-mistakes are those made by people who are perfectly competent to apply concepts, at least in the situations with which they are familiar, but are still liable in their abstract thinking to allocate those concepts to logical types to which they do not belong».</t>
         </is>
       </c>
       <c r="J185" s="7" t="n"/>
@@ -9304,7 +9304,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -9588,31 +9588,6 @@
       <c r="E11" s="7" t="inlineStr">
         <is>
           <t>Nota: «p. 27» → «pp. 27 y 28».</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="7" t="n">
-        <v>554</v>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>Pendiente (fuente no disponible)</t>
-        </is>
-      </c>
-      <c r="C12" s="7" t="inlineStr">
-        <is>
-          <t>Ibidem, p. 19.</t>
-        </is>
-      </c>
-      <c r="D12" s="7" t="inlineStr">
-        <is>
-          <t>Ryle, p. 19: el archivo subido abarca las pp. 13-18; la p. 18 termina con el ejemplo del críquet y el pasaje citado debe seguir en la p. 19, que no se recibió.</t>
-        </is>
-      </c>
-      <c r="E12" s="7" t="inlineStr">
-        <is>
-          <t>Ninguna; requiere la fuente</t>
         </is>
       </c>
     </row>
@@ -9732,7 +9707,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Pp. 13-18 subidas por el usuario (su paginación coincide con la que cita la tesis)</t>
+          <t>Pp. 13-19 enviadas por el usuario (su paginación coincide con la que cita la tesis)</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -9742,7 +9717,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Notas 552 y 553 conformes; 554 (p. 19) pendiente.</t>
+          <t>Notas 552 a 554 conformes.</t>
         </is>
       </c>
     </row>

</xml_diff>